<commit_message>
Horizonte (jun base / jul retorno) + fix ICP: backfill en cadena y jun/jul corregidos
- planilla_vc.xlsx con Horizonte; template Horizonte poblado (jun 1004.2485 base, jul 1009.8454); gate -> 2026-07.
- ICP: icp_clicp.json tenía julio mal (calc desde mayo) y sin junio; corregido secuencial (jun 26634.69, jul 26734.57). El bloque ICP ahora rellena EN CADENA todos los meses faltantes hasta el objetivo.
</commit_message>
<xml_diff>
--- a/inputs/templates/TEMPLATE FONDO LIQUIDEZ HORIZONTE.xlsx
+++ b/inputs/templates/TEMPLATE FONDO LIQUIDEZ HORIZONTE.xlsx
@@ -25,7 +25,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
@@ -35,6 +35,7 @@
     <numFmt numFmtId="170" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="171" formatCode="0.000%"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
+    <numFmt numFmtId="173" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="32">
     <font>
@@ -382,7 +383,7 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -626,6 +627,7 @@
     <xf numFmtId="169" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="29" fillId="14" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="29" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2062,7 +2064,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CL"/>
           </a:p>
@@ -2114,7 +2116,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CL"/>
           </a:p>
@@ -2199,7 +2201,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="es-CL"/>
         </a:p>
@@ -2633,7 +2635,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr lang="es-CL"/>
             </a:p>
@@ -2665,7 +2667,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CL"/>
           </a:p>
@@ -2702,7 +2704,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="es-CL"/>
         </a:p>
@@ -4027,7 +4029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK249"/>
+  <dimension ref="A1:BK252"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.28515625" defaultRowHeight="15"/>
   <cols>
     <col width="18.28515625" customWidth="1" style="14" min="1" max="2"/>
@@ -5112,7 +5114,7 @@
         </is>
       </c>
       <c r="AW19" s="84" t="n">
-        <v>46142</v>
+        <v>46203</v>
       </c>
       <c r="AX19" s="42">
         <f>EOMONTH($AW19,AX18)+6+1</f>
@@ -5389,8 +5391,14 @@
         <f>+S23/R23-1</f>
         <v/>
       </c>
-      <c r="AI22" s="20" t="n"/>
-      <c r="AJ22" s="20" t="n"/>
+      <c r="AI22" s="20">
+        <f>+T23/S23-1</f>
+        <v/>
+      </c>
+      <c r="AJ22" s="20">
+        <f>+U23/T23-1</f>
+        <v/>
+      </c>
       <c r="AK22" s="20" t="n"/>
       <c r="AL22" s="20" t="n"/>
       <c r="AM22" s="20" t="n"/>
@@ -5398,7 +5406,7 @@
       <c r="AO22" s="20" t="n"/>
       <c r="AP22" s="20" t="n"/>
       <c r="AQ22" s="34">
-        <f>+(S23/P23-1)/COUNTA(AE22:AP22)*12</f>
+        <f>+(U23/P23-1)/COUNTA(AE22:AJ22)*12</f>
         <v/>
       </c>
       <c r="AV22" s="39" t="inlineStr">
@@ -5457,7 +5465,14 @@
         <f>+B249</f>
         <v/>
       </c>
-      <c r="U23" s="30" t="n"/>
+      <c r="T23">
+        <f>+B250</f>
+        <v/>
+      </c>
+      <c r="U23" s="30">
+        <f>+B251</f>
+        <v/>
+      </c>
       <c r="Y23" s="30" t="n"/>
       <c r="AD23" s="37" t="inlineStr">
         <is>
@@ -7553,6 +7568,14 @@
         <f>+K249</f>
         <v/>
       </c>
+      <c r="T51">
+        <f>+K250</f>
+        <v/>
+      </c>
+      <c r="U51">
+        <f>+K251</f>
+        <v/>
+      </c>
       <c r="AD51" s="32" t="n">
         <v>2026</v>
       </c>
@@ -7572,8 +7595,14 @@
         <f>+(S51/R51-1)</f>
         <v/>
       </c>
-      <c r="AI51" s="20" t="n"/>
-      <c r="AJ51" s="20" t="n"/>
+      <c r="AI51" s="20">
+        <f>+T51/S51-1</f>
+        <v/>
+      </c>
+      <c r="AJ51" s="20">
+        <f>+U51/T51-1</f>
+        <v/>
+      </c>
       <c r="AK51" s="20" t="n"/>
       <c r="AL51" s="20" t="n"/>
       <c r="AM51" s="20" t="n"/>
@@ -7581,7 +7610,7 @@
       <c r="AO51" s="20" t="n"/>
       <c r="AP51" s="20" t="n"/>
       <c r="AQ51" s="34">
-        <f>+(S51/P51-1)/COUNTA(AE51:AP51)*12</f>
+        <f>+(U51/P51-1)/COUNTA(AE51:AJ51)*12</f>
         <v/>
       </c>
       <c r="AR51" s="20" t="n"/>
@@ -14382,6 +14411,98 @@
       </c>
       <c r="M249" s="30">
         <f>+M248*(1+L249)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="127" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B250" t="n">
+        <v>26535.18</v>
+      </c>
+      <c r="C250">
+        <f>(B250/B249-1)/(A250-A249)*30</f>
+        <v/>
+      </c>
+      <c r="D250">
+        <f>+D249*(1+C250)</f>
+        <v/>
+      </c>
+      <c r="F250" s="127" t="n"/>
+      <c r="K250" t="n">
+        <v>6368.94</v>
+      </c>
+      <c r="L250">
+        <f>+(K250/K249-1)/(F250-F249)*30</f>
+        <v/>
+      </c>
+      <c r="M250">
+        <f>+M249*(1+L250)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="127" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B251" t="n">
+        <v>26634.69</v>
+      </c>
+      <c r="C251">
+        <f>(B251/B250-1)/(A251-A250)*30</f>
+        <v/>
+      </c>
+      <c r="D251">
+        <f>+D250*(1+C251)</f>
+        <v/>
+      </c>
+      <c r="F251" s="127" t="n">
+        <v>46203</v>
+      </c>
+      <c r="G251" t="n">
+        <v>1004.2485</v>
+      </c>
+      <c r="H251">
+        <f>+G251</f>
+        <v/>
+      </c>
+      <c r="K251" t="n">
+        <v>6385.6713</v>
+      </c>
+      <c r="L251">
+        <f>+(K251/K250-1)/(F251-F250)*30</f>
+        <v/>
+      </c>
+      <c r="M251">
+        <f>+M250*(1+L251)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="127" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C252">
+        <f>(B252/B251-1)/(A252-A251)*30</f>
+        <v/>
+      </c>
+      <c r="D252">
+        <f>+D251*(1+C252)</f>
+        <v/>
+      </c>
+      <c r="F252" s="127" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G252" t="n">
+        <v>1009.8454</v>
+      </c>
+      <c r="H252">
+        <f>+G252</f>
+        <v/>
+      </c>
+      <c r="I252">
+        <f>+(H252/H251-1)/(F252-F251)*30</f>
         <v/>
       </c>
     </row>
@@ -14450,9 +14571,11 @@
           <t>Anual</t>
         </is>
       </c>
-      <c r="X1" s="90">
-        <f>+'Datos ICP (2)'!BB28</f>
-        <v/>
+      <c r="X1" s="90" t="inlineStr">
+        <is>
+          <t>Acum
+2026 (*)</t>
+        </is>
       </c>
     </row>
     <row r="2">

</xml_diff>